<commit_message>
Cut unresolved rows and finalize 734-entry tracker
</commit_message>
<xml_diff>
--- a/downloads/Star_Wars_Chronological_Marathon_Tracker.xlsx
+++ b/downloads/Star_Wars_Chronological_Marathon_Tracker.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marathon Tracker" sheetId="1" r:id="R1d27e39eee6b4d3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marathon Tracker" sheetId="1" r:id="Re960e50cd8e94111"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -417,7 +417,7 @@
     <x:xf numFmtId="0" fontId="8" fillId="10" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -461,7 +461,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MarathonTracker" displayName="MarathonTracker" ref="A7:S746" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MarathonTracker" displayName="MarathonTracker" ref="A7:S741" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="Done"/>
     <x:tableColumn id="2" name="#"/>
@@ -771,7 +771,7 @@
         <x:v>Rows requiring placement review</x:v>
       </x:c>
       <x:c r="H4" s="4" t="n">
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I4" s="1"/>
       <x:c r="J4" s="1"/>
@@ -814,12 +814,12 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="18" t="n">
-        <x:f>COUNTIF(A8:A746,"Yes")</x:f>
+        <x:f>COUNTIF(A8:A741,"Yes")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="B6" s="19" t="n">
-        <x:f>COUNTA(B8:B746)</x:f>
-        <x:v>739</x:v>
+        <x:f>COUNTA(B8:B741)</x:f>
+        <x:v>734</x:v>
       </x:c>
       <x:c r="C6" s="21" t="n">
         <x:f>IF(B6=0,0,A6/B6)</x:f>
@@ -931,7 +931,7 @@
         <x:v>https://www.youtube.com/results?search_query=Ancient%20Sith%20Sat%20on%20the%20Throne%20for%201%2C000%20Years</x:v>
       </x:c>
       <x:c r="K8" s="50" t="str">
-        <x:v>Generic/original Jedi, Sith, creature, or Emperor story without a dependable era anchor.; Vitiate-inspired ancient Sith story; the exact century is an estimate.</x:v>
+        <x:v>Vitiate-inspired ancient Sith story; the exact century is an estimate.</x:v>
       </x:c>
       <x:c r="L8" s="50" t="str">
         <x:v>Ancient Sith / Vitiate-inspired interlude</x:v>
@@ -39156,24 +39156,24 @@
         <x:v>LEGO alternate continuity</x:v>
       </x:c>
       <x:c r="D722" s="50" t="str">
-        <x:v>LEGO Star Wars Summer Vacation</x:v>
+        <x:v>The Freemaker Adventures</x:v>
       </x:c>
       <x:c r="E722" s="50" t="str"/>
       <x:c r="F722" s="50" t="str">
-        <x:v>August 5, 2022</x:v>
+        <x:v>June 20, 2016–August 16, 2017</x:v>
       </x:c>
       <x:c r="G722" s="50" t="str">
         <x:v>LEGO</x:v>
       </x:c>
       <x:c r="H722" s="50" t="str">
-        <x:v>Special</x:v>
+        <x:v>Series</x:v>
       </x:c>
       <x:c r="I722" s="50" t="str">
         <x:v>Disney+</x:v>
       </x:c>
       <x:c r="J722" s="50" t="str"/>
       <x:c r="K722" s="50" t="str">
-        <x:v>Post-Rise of Skywalker jumping-off point.</x:v>
+        <x:v>Original-trilogy / Age of Rebellion backdrop.</x:v>
       </x:c>
       <x:c r="L722" s="50" t="str"/>
       <x:c r="M722" s="50" t="str"/>
@@ -39273,11 +39273,11 @@
         <x:v>LEGO alternate continuity</x:v>
       </x:c>
       <x:c r="D725" s="38" t="str">
-        <x:v>LEGO Star Wars: Rebuild the Galaxy</x:v>
+        <x:v>The LEGO Star Wars Holiday Special</x:v>
       </x:c>
       <x:c r="E725" s="38" t="str"/>
       <x:c r="F725" s="38" t="str">
-        <x:v>September 13, 2024</x:v>
+        <x:v>November 17, 2020</x:v>
       </x:c>
       <x:c r="G725" s="38" t="str">
         <x:v>LEGO</x:v>
@@ -39290,7 +39290,7 @@
       </x:c>
       <x:c r="J725" s="38" t="str"/>
       <x:c r="K725" s="38" t="str">
-        <x:v>Post-Rise of Skywalker multiverse / scrambled-timeline story.</x:v>
+        <x:v>Post-Rise of Skywalker jumping-off point; time-travel alternate continuity.</x:v>
       </x:c>
       <x:c r="L725" s="38" t="str"/>
       <x:c r="M725" s="38" t="str"/>
@@ -39351,11 +39351,11 @@
         <x:v>LEGO alternate continuity</x:v>
       </x:c>
       <x:c r="D727" s="38" t="str">
-        <x:v>Rebuild the Galaxy: Pieces of the Past</x:v>
+        <x:v>LEGO Star Wars Summer Vacation</x:v>
       </x:c>
       <x:c r="E727" s="38" t="str"/>
       <x:c r="F727" s="38" t="str">
-        <x:v>September 19, 2025</x:v>
+        <x:v>August 5, 2022</x:v>
       </x:c>
       <x:c r="G727" s="38" t="str">
         <x:v>LEGO</x:v>
@@ -39368,7 +39368,7 @@
       </x:c>
       <x:c r="J727" s="38" t="str"/>
       <x:c r="K727" s="38" t="str">
-        <x:v>Continuation of Rebuild the Galaxy.</x:v>
+        <x:v>Post-Rise of Skywalker jumping-off point.</x:v>
       </x:c>
       <x:c r="L727" s="38" t="str"/>
       <x:c r="M727" s="38" t="str"/>
@@ -39390,24 +39390,24 @@
         <x:v>LEGO alternate continuity</x:v>
       </x:c>
       <x:c r="D728" s="38" t="str">
-        <x:v>The Freemaker Adventures</x:v>
+        <x:v>LEGO Star Wars: Rebuild the Galaxy</x:v>
       </x:c>
       <x:c r="E728" s="38" t="str"/>
       <x:c r="F728" s="38" t="str">
-        <x:v>June 20, 2016–August 16, 2017</x:v>
+        <x:v>September 13, 2024</x:v>
       </x:c>
       <x:c r="G728" s="38" t="str">
         <x:v>LEGO</x:v>
       </x:c>
       <x:c r="H728" s="38" t="str">
-        <x:v>Series</x:v>
+        <x:v>Special</x:v>
       </x:c>
       <x:c r="I728" s="38" t="str">
         <x:v>Disney+</x:v>
       </x:c>
       <x:c r="J728" s="38" t="str"/>
       <x:c r="K728" s="38" t="str">
-        <x:v>Original-trilogy / Age of Rebellion backdrop.</x:v>
+        <x:v>Post-Rise of Skywalker multiverse / scrambled-timeline story.</x:v>
       </x:c>
       <x:c r="L728" s="38" t="str"/>
       <x:c r="M728" s="38" t="str"/>
@@ -39429,11 +39429,11 @@
         <x:v>LEGO alternate continuity</x:v>
       </x:c>
       <x:c r="D729" s="38" t="str">
-        <x:v>The LEGO Star Wars Holiday Special</x:v>
+        <x:v>Rebuild the Galaxy: Pieces of the Past</x:v>
       </x:c>
       <x:c r="E729" s="38" t="str"/>
       <x:c r="F729" s="38" t="str">
-        <x:v>November 17, 2020</x:v>
+        <x:v>September 19, 2025</x:v>
       </x:c>
       <x:c r="G729" s="38" t="str">
         <x:v>LEGO</x:v>
@@ -39446,7 +39446,7 @@
       </x:c>
       <x:c r="J729" s="38" t="str"/>
       <x:c r="K729" s="38" t="str">
-        <x:v>Post-Rise of Skywalker jumping-off point; time-travel alternate continuity.</x:v>
+        <x:v>Continuation of Rebuild the Galaxy.</x:v>
       </x:c>
       <x:c r="L729" s="38" t="str"/>
       <x:c r="M729" s="38" t="str"/>
@@ -39889,392 +39889,64 @@
       <x:c r="S740" s="38" t="str"/>
     </x:row>
     <x:row r="741" ht="42" customHeight="1">
-      <x:c r="A741" s="44" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="B741" s="44" t="n">
+      <x:c r="A741" s="45" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="B741" s="45" t="n">
         <x:v>734</x:v>
       </x:c>
-      <x:c r="C741" s="64" t="str">
+      <x:c r="C741" s="70" t="str">
         <x:v>Abandoned and reconstructed stories</x:v>
       </x:c>
-      <x:c r="D741" s="38" t="str">
+      <x:c r="D741" s="39" t="str">
         <x:v>Mr Sunday Movies animated summary</x:v>
       </x:c>
-      <x:c r="E741" s="38" t="str"/>
-      <x:c r="F741" s="38" t="str">
+      <x:c r="E741" s="39" t="str"/>
+      <x:c r="F741" s="39" t="str">
         <x:v>2020</x:v>
       </x:c>
-      <x:c r="G741" s="38" t="str">
+      <x:c r="G741" s="39" t="str">
         <x:v>Fan / non-canon</x:v>
       </x:c>
-      <x:c r="H741" s="38" t="str">
+      <x:c r="H741" s="39" t="str">
         <x:v>Animated summary</x:v>
       </x:c>
-      <x:c r="I741" s="38" t="str">
+      <x:c r="I741" s="39" t="str">
         <x:v>YouTube</x:v>
       </x:c>
-      <x:c r="J741" s="38" t="str">
+      <x:c r="J741" s="39" t="str">
         <x:v>https://www.youtube.com/watch?v=9WEU1b2t1zM</x:v>
       </x:c>
-      <x:c r="K741" s="38" t="str"/>
-      <x:c r="L741" s="38" t="str"/>
-      <x:c r="M741" s="38" t="str"/>
-      <x:c r="N741" s="38" t="str"/>
-      <x:c r="O741" s="38" t="str"/>
-      <x:c r="P741" s="38" t="str"/>
-      <x:c r="Q741" s="38" t="str"/>
-      <x:c r="R741" s="38" t="str"/>
-      <x:c r="S741" s="38" t="str"/>
-    </x:row>
-    <x:row r="742" ht="42" customHeight="1">
-      <x:c r="A742" s="48" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="B742" s="48" t="n">
-        <x:v>735</x:v>
-      </x:c>
-      <x:c r="C742" s="69" t="str">
-        <x:v>Unplaced fan stories — review and decide</x:v>
-      </x:c>
-      <x:c r="D742" s="50" t="str">
-        <x:v>4 The Storm Beast Awakens 4</x:v>
-      </x:c>
-      <x:c r="E742" s="50" t="str"/>
-      <x:c r="F742" s="50" t="str">
-        <x:v>June 11, 2026</x:v>
-      </x:c>
-      <x:c r="G742" s="50" t="str">
-        <x:v>Fan-made / non-canon</x:v>
-      </x:c>
-      <x:c r="H742" s="50" t="str">
-        <x:v>Fan video</x:v>
-      </x:c>
-      <x:c r="I742" s="50" t="str">
-        <x:v>YouTube — search by title</x:v>
-      </x:c>
-      <x:c r="J742" s="50" t="str">
-        <x:v>https://www.youtube.com/results?search_query=4%20The%20Storm%20Beast%20Awakens%204</x:v>
-      </x:c>
-      <x:c r="K742" s="50" t="str">
-        <x:v>Generic/original Jedi, Sith, creature, or Emperor story without a dependable era anchor.</x:v>
-      </x:c>
-      <x:c r="L742" s="50" t="str">
-        <x:v>Below timeline — era not stated</x:v>
-      </x:c>
-      <x:c r="M742" s="50" t="str"/>
-      <x:c r="N742" s="50" t="str">
-        <x:v>The sky darkens without warning. Thunder shakes
-the mountains as an ancient Storm Beast rises from
-the heart of the tempest. Lightning crashes around
-a lone Jedi who must face a creature powered by
-the fury of the storm itself. Every strike lights up the
-battlefield as the Force clashes with the raw power
-of nature.
-™ One Jedi.
-4 One Storm Beast.
-@ One battle that will shake the heavens.
-#jedi #stormbeast #theforce #lightsaber
-#epicbattle #fantasy #legendary #storm #thunder
-#cinematic #viral #fyp #tiktok #adventure
-#forcebattle</x:v>
-      </x:c>
-      <x:c r="O742" s="50" t="str">
-        <x:v>IMG_6630.PNG</x:v>
-      </x:c>
-      <x:c r="P742" s="50" t="str">
-        <x:v>Needs review</x:v>
-      </x:c>
-      <x:c r="Q742" s="50" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="R742" s="50" t="str">
-        <x:v>No named character, faction, or dated event is visible; retained below the timeline rather than guessed.</x:v>
-      </x:c>
-      <x:c r="S742" s="50" t="str">
-        <x:v>Unique</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="743" ht="42" customHeight="1">
-      <x:c r="A743" s="44" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="B743" s="44" t="n">
-        <x:v>736</x:v>
-      </x:c>
-      <x:c r="C743" s="67" t="str">
-        <x:v>Unplaced fan stories — review and decide</x:v>
-      </x:c>
-      <x:c r="D743" s="38" t="str">
-        <x:v>The Huntress on the Train</x:v>
-      </x:c>
-      <x:c r="E743" s="38" t="str"/>
-      <x:c r="F743" s="38" t="str">
-        <x:v>August 22, 2026</x:v>
-      </x:c>
-      <x:c r="G743" s="38" t="str">
-        <x:v>Fan-made / non-canon</x:v>
-      </x:c>
-      <x:c r="H743" s="38" t="str">
-        <x:v>Fan video</x:v>
-      </x:c>
-      <x:c r="I743" s="38" t="str">
-        <x:v>YouTube — search by title</x:v>
-      </x:c>
-      <x:c r="J743" s="38" t="str">
-        <x:v>https://www.youtube.com/results?search_query=The%20Huntress%20on%20the%20Train</x:v>
-      </x:c>
-      <x:c r="K743" s="38" t="str">
-        <x:v>No reliable canonical or Legends-era anchor is stated; user decision required.</x:v>
-      </x:c>
-      <x:c r="L743" s="38" t="str">
-        <x:v>Unplaced original Huntress continuity</x:v>
-      </x:c>
-      <x:c r="M743" s="38" t="str"/>
-      <x:c r="N743" s="38" t="str">
-        <x:v>3 Cash App: $brednew
-© PayPal: @blainehenry688
-The Huntress races across the top of a speeding
-train with her blue and green lightsabers blazing.
-One wrong move and it's over.
-But slowing down was never an option.
-#TheHuntress #Lightsaber #Jedi #Cinematic
-#StarWars
-How this was made
-Made with Al
-Sounds or visuals were altered or fully generated. Learn</x:v>
-      </x:c>
-      <x:c r="O743" s="38" t="str">
-        <x:v>IMG_6583.PNG</x:v>
-      </x:c>
-      <x:c r="P743" s="38" t="str">
-        <x:v>Needs review</x:v>
-      </x:c>
-      <x:c r="Q743" s="38" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="R743" s="38" t="str">
-        <x:v>The blue-and-green-lightsaber Huntress shown here is not identified as Darth Cognus, and the visible description gives no galactic era.</x:v>
-      </x:c>
-      <x:c r="S743" s="38" t="str">
-        <x:v>Unique</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="744" ht="42" customHeight="1">
-      <x:c r="A744" s="44" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="B744" s="44" t="n">
-        <x:v>737</x:v>
-      </x:c>
-      <x:c r="C744" s="67" t="str">
-        <x:v>Unplaced fan stories — review and decide</x:v>
-      </x:c>
-      <x:c r="D744" s="38" t="str">
-        <x:v>The Huntress Will Return | Nothing Can Stop Her</x:v>
-      </x:c>
-      <x:c r="E744" s="38" t="str"/>
-      <x:c r="F744" s="38" t="str">
-        <x:v>August 23, 2026</x:v>
-      </x:c>
-      <x:c r="G744" s="38" t="str">
-        <x:v>Fan-made / non-canon</x:v>
-      </x:c>
-      <x:c r="H744" s="38" t="str">
-        <x:v>Fan video</x:v>
-      </x:c>
-      <x:c r="I744" s="38" t="str">
-        <x:v>YouTube — search by title</x:v>
-      </x:c>
-      <x:c r="J744" s="38" t="str">
-        <x:v>https://www.youtube.com/results?search_query=The%20Huntress%20Will%20Return%20%7C%20Nothing%20Can%20Stop%20Her</x:v>
-      </x:c>
-      <x:c r="K744" s="38" t="str">
-        <x:v>No reliable canonical or Legends-era anchor is stated; user decision required.</x:v>
-      </x:c>
-      <x:c r="L744" s="38" t="str">
-        <x:v>Unplaced original Huntress continuity</x:v>
-      </x:c>
-      <x:c r="M744" s="38" t="str"/>
-      <x:c r="N744" s="38" t="str">
-        <x:v>3 Cash App: $brednew
-© PayPal: @blainehenry688
-They opened fire.
-The Huntress kept coming.
-With her signature BLUE and GREEN lightsabers,
-she charges straight through a storm of blaster fire
-without slowing down.
-And this battle isn't the end.
-THE HUNTRESS WILL RETURN.
-#TheHuntress #Jedi #Lightsaber #StarWars
-#StarWarsLore #Cinematic</x:v>
-      </x:c>
-      <x:c r="O744" s="38" t="str">
-        <x:v>IMG_6574.PNG</x:v>
-      </x:c>
-      <x:c r="P744" s="38" t="str">
-        <x:v>Needs review</x:v>
-      </x:c>
-      <x:c r="Q744" s="38" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="R744" s="38" t="str">
-        <x:v>The blue-and-green-lightsaber Huntress shown here is not identified as Darth Cognus, and the visible description gives no galactic era.</x:v>
-      </x:c>
-      <x:c r="S744" s="38" t="str">
-        <x:v>Unique</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="745" ht="42" customHeight="1">
-      <x:c r="A745" s="44" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="B745" s="44" t="n">
-        <x:v>738</x:v>
-      </x:c>
-      <x:c r="C745" s="67" t="str">
-        <x:v>Unplaced fan stories — review and decide</x:v>
-      </x:c>
-      <x:c r="D745" s="38" t="str">
-        <x:v>The Huntress: When Hope Falls... Legends Rise</x:v>
-      </x:c>
-      <x:c r="E745" s="38" t="str"/>
-      <x:c r="F745" s="38" t="str">
-        <x:v>August 23, 2026</x:v>
-      </x:c>
-      <x:c r="G745" s="38" t="str">
-        <x:v>Fan-made / non-canon</x:v>
-      </x:c>
-      <x:c r="H745" s="38" t="str">
-        <x:v>Fan video</x:v>
-      </x:c>
-      <x:c r="I745" s="38" t="str">
-        <x:v>YouTube — search by title</x:v>
-      </x:c>
-      <x:c r="J745" s="38" t="str">
-        <x:v>https://www.youtube.com/results?search_query=The%20Huntress%3A%20When%20Hope%20Falls...%20Legends%20Rise</x:v>
-      </x:c>
-      <x:c r="K745" s="38" t="str">
-        <x:v>No reliable canonical or Legends-era anchor is stated; user decision required.</x:v>
-      </x:c>
-      <x:c r="L745" s="38" t="str">
-        <x:v>Unplaced original Huntress continuity</x:v>
-      </x:c>
-      <x:c r="M745" s="38" t="str"/>
-      <x:c r="N745" s="38" t="str">
-        <x:v>3 Cash App: $brednew
-© PayPal: @blainehenry688
-The city is falling. Chaos has taken the streets.
-Everyone is running from the danger.
-Except the Huntress.
-With her signature BLUE and GREEN lightsabers,
-she moves straight into the fight. When everything
-begins to collapse, some warriors don’t retreat.
-When hope falls... legends rise.
-#TheHuntress #Jedi #Lightsaber #StarWars
-#StarWarsLore #Cinematic</x:v>
-      </x:c>
-      <x:c r="O745" s="38" t="str">
-        <x:v>IMG_6577.PNG</x:v>
-      </x:c>
-      <x:c r="P745" s="38" t="str">
-        <x:v>Needs review</x:v>
-      </x:c>
-      <x:c r="Q745" s="38" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="R745" s="38" t="str">
-        <x:v>The blue-and-green-lightsaber Huntress shown here is not identified as Darth Cognus, and the visible description gives no galactic era.</x:v>
-      </x:c>
-      <x:c r="S745" s="38" t="str">
-        <x:v>Unique</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="746" ht="42" customHeight="1">
-      <x:c r="A746" s="45" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="B746" s="45" t="n">
-        <x:v>739</x:v>
-      </x:c>
-      <x:c r="C746" s="70" t="str">
-        <x:v>Unplaced fan stories — review and decide</x:v>
-      </x:c>
-      <x:c r="D746" s="39" t="str">
-        <x:v>They Surrounded the Huntress — That Was Their Mistake</x:v>
-      </x:c>
-      <x:c r="E746" s="39" t="str"/>
-      <x:c r="F746" s="39" t="str">
-        <x:v>August 20, 2026</x:v>
-      </x:c>
-      <x:c r="G746" s="39" t="str">
-        <x:v>Fan-made / non-canon</x:v>
-      </x:c>
-      <x:c r="H746" s="39" t="str">
-        <x:v>Fan video</x:v>
-      </x:c>
-      <x:c r="I746" s="39" t="str">
-        <x:v>YouTube — search by title</x:v>
-      </x:c>
-      <x:c r="J746" s="39" t="str">
-        <x:v>https://www.youtube.com/results?search_query=They%20Surrounded%20the%20Huntress%20%E2%80%94%20That%20Was%20Their%20Mistake</x:v>
-      </x:c>
-      <x:c r="K746" s="39" t="str">
-        <x:v>No reliable canonical or Legends-era anchor is stated; user decision required.</x:v>
-      </x:c>
-      <x:c r="L746" s="39" t="str">
-        <x:v>Unplaced original Huntress continuity</x:v>
-      </x:c>
-      <x:c r="M746" s="39" t="str"/>
-      <x:c r="N746" s="39" t="str">
-        <x:v>i Cash App: $brednew
-© PayPal: @blainehenry688
-é SUPPORT THE CHANNEL @&amp;
-Even 5¢, 10¢, 25¢, or $1 helps us continue creating
-these cinematic stories and building this universe.
-The Huntress walks straight into a battlefield
-crawling with enemy soldiers.
-Outnumbered and surrounded, she doesn't retreat.
-She draws her lightsabers and stands her ground as
-another Jedi joins the fight beside her.
-For most warriors, being surrounded means you're</x:v>
-      </x:c>
-      <x:c r="O746" s="39" t="str">
-        <x:v>IMG_6749.PNG</x:v>
-      </x:c>
-      <x:c r="P746" s="39" t="str">
-        <x:v>Needs review</x:v>
-      </x:c>
-      <x:c r="Q746" s="39" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="R746" s="39" t="str">
-        <x:v>The blue-and-green-lightsaber Huntress shown here is not identified as Darth Cognus, and the visible description gives no galactic era.</x:v>
-      </x:c>
-      <x:c r="S746" s="39" t="str">
-        <x:v>Unique</x:v>
-      </x:c>
+      <x:c r="K741" s="39" t="str"/>
+      <x:c r="L741" s="39" t="str"/>
+      <x:c r="M741" s="39" t="str"/>
+      <x:c r="N741" s="39" t="str"/>
+      <x:c r="O741" s="39" t="str"/>
+      <x:c r="P741" s="39" t="str"/>
+      <x:c r="Q741" s="39" t="str"/>
+      <x:c r="R741" s="39" t="str"/>
+      <x:c r="S741" s="39" t="str"/>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="A8:S746">
+  <x:conditionalFormatting sqref="A8:S741">
     <x:cfRule type="expression" dxfId="0" priority="1">
       <x:formula>$A8="Yes"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="Q8:Q746">
+  <x:conditionalFormatting sqref="Q8:Q741">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Low"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="R8:R746">
+  <x:conditionalFormatting sqref="R8:R741">
     <x:cfRule type="notContainsBlanks" dxfId="2" priority="3"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="A8:A746">
+    <x:dataValidation type="list" sqref="A8:A741">
       <x:formula1>"No,Yes"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e98ca334b7545ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99c010fca9674c15"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>